<commit_message>
Updated POL_grids_kan50 model - 2026-08-28 17:17
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5CA49BAF-899E-4189-B0E1-3560A50A9572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD480F00-20BA-4B67-A9B4-A4A8216EC516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="70" r:id="rId1"/>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360840F2-9C18-4BE0-83CC-7DF4419CB0FF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F947EE5-BC23-4944-BE05-3606B8840C8D}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3C937D4-6DA5-4FE2-8F4F-DE4705BF8074}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEF167F-2F6D-4727-A621-40E99730D4C5}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-08-28 18:08
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD480F00-20BA-4B67-A9B4-A4A8216EC516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17812D27-E688-4818-823B-35681B340D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F947EE5-BC23-4944-BE05-3606B8840C8D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C27D89FD-F1D5-460D-8FED-89352FFB136E}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEF167F-2F6D-4727-A621-40E99730D4C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D03BCF45-6FB6-4F6D-92D1-57F45CB4E2D1}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-08-28 22:33
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17812D27-E688-4818-823B-35681B340D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11BAEB3-8007-45C2-A56D-405E59881DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C27D89FD-F1D5-460D-8FED-89352FFB136E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2279353-07CF-47A0-9CEE-F57D2F58F5E3}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D03BCF45-6FB6-4F6D-92D1-57F45CB4E2D1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC8FDAA-075D-4916-AD4A-943EEA3F3ED1}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-08-29 12:15
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11BAEB3-8007-45C2-A56D-405E59881DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4AD272-80F7-491C-B23C-8A899500C7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2279353-07CF-47A0-9CEE-F57D2F58F5E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BEDC9A-6CDB-41A1-B249-3C817DF74DCE}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EC8FDAA-075D-4916-AD4A-943EEA3F3ED1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD355335-0B1F-4159-9FD3-FB0E4C2C8352}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-08-29 13:03
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4AD272-80F7-491C-B23C-8A899500C7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E029F6C1-7E21-4538-87A2-C815E9F86834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BEDC9A-6CDB-41A1-B249-3C817DF74DCE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53AA1E5-116F-4543-B0C4-945A73A77409}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD355335-0B1F-4159-9FD3-FB0E4C2C8352}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C564CFC8-8FA5-4255-B2B4-FF62B679F93B}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-08-30 20:55
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE6C06E8-D9F0-4F31-9C1B-91A8C8C796D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC3A58EA-4490-422F-9000-401DC32F357B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39593520-9087-4260-8706-424D8764DA25}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A458DBB-6C0A-4B6E-A8B8-F98B0C398097}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{992286AE-3905-4A46-9913-55C5FAD78205}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EF339BF-497D-4250-BF1F-205660B0FF48}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-09-03 16:23
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC3A58EA-4490-422F-9000-401DC32F357B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3134D195-60F9-4F88-A98A-498DB012409D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3681,7 +3681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A458DBB-6C0A-4B6E-A8B8-F98B0C398097}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD4708C-6F46-4059-BFF7-5B8B8352995B}">
   <dimension ref="B9:L186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -31401,7 +31401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EF339BF-497D-4250-BF1F-205660B0FF48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A9FCB23-BE29-496D-B49D-AC1087386603}">
   <dimension ref="B9:H186"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>